<commit_message>
Update Machine model, Andon authorization logic, and Swagger documentation
</commit_message>
<xml_diff>
--- a/prisma/csv/data_master_masalah_andon.xlsx
+++ b/prisma/csv/data_master_masalah_andon.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Projects\0Magang\Toshin-Backend\prisma\csv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PT. Toshin Prima\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69FB7C09-A976-447D-905F-004EA3823A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1254DAF4-F893-4E7E-B5EB-562C0F424755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MAINTENANCE" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="28">
   <si>
     <t>No</t>
   </si>
@@ -38,45 +38,12 @@
     <t>Breakdown MNT</t>
   </si>
   <si>
-    <t>00:55:00</t>
-  </si>
-  <si>
-    <t>Preventive MNT</t>
-  </si>
-  <si>
     <t>00:05:00</t>
   </si>
   <si>
-    <t>Corrective MNT</t>
-  </si>
-  <si>
-    <t>01:00:00</t>
-  </si>
-  <si>
-    <t>Improvement</t>
-  </si>
-  <si>
-    <t>Replace Part</t>
-  </si>
-  <si>
-    <t>00:30:00</t>
-  </si>
-  <si>
-    <t>Cleaning</t>
-  </si>
-  <si>
     <t>00:15:00</t>
   </si>
   <si>
-    <t>Ganti Silinder Invit</t>
-  </si>
-  <si>
-    <t>Minor Stop Invit</t>
-  </si>
-  <si>
-    <t>00:20:00</t>
-  </si>
-  <si>
     <t>Initial Check</t>
   </si>
   <si>
@@ -101,45 +68,9 @@
     <t>00:45:00</t>
   </si>
   <si>
-    <t>Setup Dies</t>
-  </si>
-  <si>
-    <t>Unsetup Dies</t>
-  </si>
-  <si>
-    <t>Setup Coil</t>
-  </si>
-  <si>
-    <t>Unsetup Coil</t>
-  </si>
-  <si>
-    <t>00:10:00</t>
-  </si>
-  <si>
     <t>Ganti Bak Scrap</t>
   </si>
   <si>
-    <t>Setting Nozzle</t>
-  </si>
-  <si>
-    <t>Die Safety</t>
-  </si>
-  <si>
-    <t>Isi Cutting Oil</t>
-  </si>
-  <si>
-    <t>00:03:00</t>
-  </si>
-  <si>
-    <t>Stp Unsetup Ds</t>
-  </si>
-  <si>
-    <t>00:25:00</t>
-  </si>
-  <si>
-    <t>Stp Unsetup CL</t>
-  </si>
-  <si>
     <t>Trial Produk</t>
   </si>
   <si>
@@ -168,12 +99,24 @@
   </si>
   <si>
     <t>Pindah Jenis Pekerjaan</t>
+  </si>
+  <si>
+    <t>sesuai obrolan kemaren sebelum checkout dikasih keterangan, jenis breakdown .....</t>
+  </si>
+  <si>
+    <t>Dandori Dies</t>
+  </si>
+  <si>
+    <t>Dandori Coil</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="166" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -203,12 +146,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -513,10 +460,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="22.1328125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -527,94 +477,23 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>15</v>
-      </c>
-      <c r="C9" t="s">
-        <v>16</v>
-      </c>
-    </row>
+      <c r="C2" s="3">
+        <v>2.0833333333333332E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="7.15" customHeight="1" x14ac:dyDescent="0.45"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -623,9 +502,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="15.9296875" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -636,37 +518,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3">
+        <v>1.3888888888888889E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -677,9 +559,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="22" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -690,37 +575,37 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -730,10 +615,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:C12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="2" max="2" width="23.59765625" customWidth="1"/>
+    <col min="3" max="3" width="19.265625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -744,125 +633,48 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="C4" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A6">
-        <v>5</v>
-      </c>
-      <c r="B6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A8">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A11">
-        <v>10</v>
-      </c>
-      <c r="B11" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A12">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>38</v>
-      </c>
-      <c r="C12" t="s">
-        <v>36</v>
+        <v>15</v>
+      </c>
+      <c r="C5" s="4">
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
   </sheetData>
@@ -873,13 +685,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77BF2988-98CD-4D20-B3E9-6467B8190619}">
   <dimension ref="A1:C10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="42" customWidth="1"/>
-    <col min="3" max="3" width="36.81640625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="36.796875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -890,100 +702,100 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>39</v>
+        <v>16</v>
       </c>
       <c r="C2" s="2">
         <v>2.0833333333333333E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>41</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>42</v>
+        <v>19</v>
       </c>
       <c r="C5" s="2">
         <v>6.9444444444444447E-4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>43</v>
+        <v>20</v>
       </c>
       <c r="C6" s="2">
         <v>1.0416666666666666E-2</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>21</v>
       </c>
       <c r="C7" s="2">
         <v>2.0833333333333333E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="C8" s="2">
         <v>2.0833333333333333E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="C9" s="2">
         <v>3.472222222222222E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>47</v>
+        <v>24</v>
       </c>
       <c r="C10" s="2">
         <v>6.9444444444444441E-3</v>

</xml_diff>